<commit_message>
Add complex-check examples: aggregate controls and excel-driven rules suite
- hop-1 Controls: count_distinct/null_count/sum/max plus CUPERS-grouped
  count on the landed table, certified by phase1_hop1_trailer.csv
- data/rules/phase1_complex_rules.xlsx (via generate_phase1_rules.py):
  11 rules exercising CUSTOM_SQL inner selects (GROUP BY/HAVING,
  correlated EXISTS and COUNT), multi-file source joins verified against
  v_dim_customer_src, differing-key LOOKUP, CUSTOM_PYTHON defaults and
  cross-file watermark consistency
- tests/migration/10_business_rules.robot: opt-in via -v RULES_WORKBOOK
  so hop-2/3 runs of tests/migration skip cleanly
- controls._dec now rejects non-finite decimals: a nullable CSV numeric
  column poisoned sum() with NaN, producing spurious control mismatches

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/phase1_hop1_csv_to_stage.xlsx
+++ b/data/mapping/phase1_hop1_csv_to_stage.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -455,15 +455,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>against cup00301, and certified row counts vs phase1_hop1_trailer.csv.</t>
+          <t>against cup00301, and certified aggregates vs phase1_hop1_trailer.csv:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>row counts, distinct keys, tax-id nulls, NAICS sum, max country code,</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>and the per-customer-type (CUPERS) grouped count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Direct copies only — all transformation happens at hop 2 per spec.</t>
         </is>
@@ -1732,7 +1746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1854,6 +1868,151 @@
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>csv_cup00301</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cup00301_distinct_cunbr</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>count_distinct</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>csv_cup00301</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cup00301_taxid_nulls</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>null_count</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cussnr</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>csv_cup00301</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>cup00301_naics_sum</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>cusic</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>csv_cup00301</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>cup00301_max_country</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>cucncd</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>csv_cup00301</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cup00301_by_pers</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>cupers</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
Consolidate validation into one end-to-end suite with traceability layer
Single input template (mapping workbook incl. Rules sheet with plain-English
Business Rule text), single suite (01_end_to_end_migration_testing — five
ordered lifecycle tests), single consolidated report (end_to_end_summary.xlsx
+ end_to_end_report.md with reviewer sheets and QA diagnostics). Requirement
IDs flow workbook -> contract -> evidence into rtm.xlsx, the DC/DA/DI/DG
compliance_scorecard, and failure-only defect_report.md. Adds test-plan
generator, Devin playbook, hop-2 BR-BIRTHDT-ISO rule; removes per-stage
suites 01_-10_ and the standalone rules workbook.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/phase1_hop1_csv_to_stage.xlsx
+++ b/data/mapping/phase1_hop1_csv_to_stage.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -504,6 +505,44 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>Direct copies only — all transformation happens at hop 2 per spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rules sheet: 11 complex business rules (aggregation via inner select,</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>correlated EXISTS, multi-file joins, lookup + default logic, format</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>checks) run by the end-to-end lifecycle suite — this workbook is the single</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>input template. 'Business Rule' columns explain each rule in plain</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>English (documentation only — not executed).</t>
         </is>
       </c>
     </row>
@@ -518,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,6 +611,11 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -616,6 +660,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>REQ-DC-101</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -660,6 +709,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>REQ-DC-102</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -702,6 +756,11 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>REQ-DC-103</t>
         </is>
       </c>
     </row>
@@ -716,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -770,6 +829,16 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Business Rule</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -810,6 +879,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -854,6 +929,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -898,6 +979,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -938,6 +1025,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -978,6 +1071,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1022,6 +1121,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1066,6 +1171,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1110,6 +1221,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1154,6 +1271,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1198,6 +1321,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1242,6 +1371,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1286,6 +1421,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1330,6 +1471,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1374,6 +1521,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1418,6 +1571,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1462,6 +1621,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1502,6 +1667,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1546,6 +1717,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1590,6 +1767,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1630,6 +1813,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1674,6 +1863,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1718,6 +1913,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1758,6 +1959,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1802,6 +2009,12 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>direct copy</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1814,7 +2027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1853,6 +2066,11 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1882,6 +2100,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>REQ-DC-101</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1911,6 +2134,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>REQ-DC-102</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1940,6 +2168,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>REQ-DC-103</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1969,6 +2202,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>REQ-DI-101</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1998,6 +2236,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>REQ-DC-104</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2027,6 +2270,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>REQ-DA-101</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2056,6 +2304,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>REQ-DA-102</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2083,6 +2336,11 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>REQ-DA-103</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2126,6 +2384,11 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2151,6 +2414,11 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>REQ-DI-102</t>
         </is>
       </c>
     </row>
@@ -2188,4 +2456,735 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Rule Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Source Table</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Source Column(s)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Target Table</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Transformation Logic</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Where Clause</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Key Column</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Business Rule</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BR-AGG-UNIQ-CUNBR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CUSTOM_SQL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>cup00301</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>cunbr IN (SELECT cunbr FROM signature.cup00301 GROUP BY cunbr HAVING COUNT(*) = 1)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>customer number must be unique across the landed customer table</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>REQ-DI-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BR-AGG-BANK-CAP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CUSTOM_SQL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>cup00301</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>cubk</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(SELECT COUNT(*) FROM signature.cup00301 x WHERE x.cubk = cup00301.cubk) &lt;= 80</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>no single bank may supply more than 80 landed customers</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>REQ-DA-104</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BR-FK-CUNBR-EXISTS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CUSTOM_SQL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>cup01201</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>EXISTS (SELECT 1 FROM signature.cup00301 p WHERE p.cunbr = cup01201.cunbr)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>every legal-entity row must reference a customer that landed</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>REQ-DI-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BR-TAXID-FORMAT</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CUSTOM_SQL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cup00301</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>cussnr</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>cussty IS NULL OR cussty &lt;&gt; 'S' OR cussnr IS NULL OR cussnr ~ '^[0-9]{9}$'</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>tax ids declared as SSN-type ('S') must be exactly 9 digits when present</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>REQ-DI-104</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BR-JOIN-LEGAL-ENTITY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DIRECT_COMPARE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>cup00301, cup01201</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>culegenty</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>v_dim_customer_src</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>culegenty</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>legal-entity code in the join view must match the CUP01201 extract per customer</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>REQ-DA-105</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BR-LOOKUP-TAXID-DESC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LOOKUP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cup00301, dim_reference@cussty=attribute_cd</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>v_dim_customer_src</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>attribute_value_desc</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>lookup(attribute_value_desc)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>cussty IS NOT NULL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>tax-id-type description must match the DIM_REFERENCE decode for declared types</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>REQ-DA-106</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BR-DEFAULT-TAXID-DESC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CUSTOM_PYTHON</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cup00301, cup01201, dim_reference@cussty=attribute_cd</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>v_dim_customer_src</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>attribute_value_desc</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>attribute_value_desc if attribute_value_desc is not None else 'SOCIAL SECURITY NUMBER'</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>a blank tax-id type decodes to 'SOCIAL SECURITY NUMBER' (spec default)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>REQ-DA-106</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BR-EXTRACT-CUT-DATE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CUSTOM_PYTHON</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>cup00301, cup01201</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>load_date</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>cup01201</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>load_date</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>load_date</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>legal-entity extract cut date must equal the customer extract cut date</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>REQ-DC-105</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BR-STATE-FORMAT</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>REGEX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>cup00301</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>cuadst</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>^[A-Z]{2}$</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>state code must be two uppercase letters</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>REQ-DI-105</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BR-JOBDATE-FORMAT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DATE_FORMAT</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>cup00301</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>cujbdt</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>%Y%m%d</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>birth date must be a valid 8-digit YYYYMMDD value</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>REQ-DI-106</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BR-SCOPED-NOTNULL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NULL_CHECK</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>cup01201</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>culegenty</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>EXISTS (SELECT 1 FROM signature.cup00301 c WHERE c.cunbr = cup01201.cunbr)</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>cunbr</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>legal-entity rows whose customer landed must have a non-null entity type</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>REQ-DI-107</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add plain-English descriptions for field mappings and business rules
Reviewers no longer have to decode engine expressions or SQL predicates:
every FieldMap row and every rule carries a Description column rendered
next to the logic in migration_report.pdf, migration_summary.xlsx,
business_rules_summary.xlsx and migration_report.md (e.g. "customer
number must be unique across the landed customer table").

Also fixes the Business rules section never reaching the PDF: the rules
suite imports ReconciliationLibrary by file path, so its instance is not
resolvable from other suites' teardowns. Write Rules Summary now drops a
rules_results.json sidecar that write_migration_pdf picks up from the
output directory, and the rules suite teardown refreshes the migration
evidence when a migration run is in progress.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/phase1_hop1_csv_to_stage.xlsx
+++ b/data/mapping/phase1_hop1_csv_to_stage.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,6 +572,11 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source Tables</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -616,6 +621,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -660,6 +666,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -704,6 +711,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -716,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -770,6 +778,11 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -810,6 +823,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Bank code - loaded unchanged</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -854,6 +872,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Customer number - the record key</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -896,6 +919,11 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Person/organization flag</t>
         </is>
       </c>
     </row>
@@ -938,6 +966,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Country code</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -978,6 +1011,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>NAICS industry code</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1022,6 +1060,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Customer name (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1066,6 +1109,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>First name (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1110,6 +1158,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Last name (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1154,6 +1207,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Tax id / SSN (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1198,6 +1256,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Tax id type code</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1242,6 +1305,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Birth/job date as YYYYMMDD</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1286,6 +1354,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Address line 1 (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1330,6 +1403,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Address line 2 (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1374,6 +1452,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>City (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1418,6 +1501,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>State code (PII)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1460,6 +1548,11 @@
       <c r="J17" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Postal code (PII)</t>
         </is>
       </c>
     </row>
@@ -1502,6 +1595,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Extract load date</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1546,6 +1644,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Customer number - links to cup00301</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1588,6 +1691,11 @@
       <c r="J20" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Legal entity code</t>
         </is>
       </c>
     </row>
@@ -1630,6 +1738,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Extract load date</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1674,6 +1787,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Reference attribute code (key)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1716,6 +1834,11 @@
       <c r="J23" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Reference value description</t>
         </is>
       </c>
     </row>
@@ -1758,6 +1881,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Extract load date</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1800,6 +1928,11 @@
       <c r="J25" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Lookup key used by category joins</t>
         </is>
       </c>
     </row>

</xml_diff>